<commit_message>
Sync package with revised manuscript: appendix renumbering and Table 4 text
- Appendix tables renumbered to match the manuscript: coverage-bar
  sensitivity is now Table A6 (tableA6_h3_bar_sensitivity), crisis-type
  heterogeneity is now Table A7 (tableA7_crisis_type_heterogeneity).
  Updated generate_tables.py, 99_validate.py, 00_run_all.py, both
  manifests, expected_final_results.csv, and script docstrings.
- Table 4 rebuilt to the manuscript's revised wording, row order, and
  "Verdict" column; every number is still interpolated from result files.
- Budget-deadline wording (docstring, DATA_CONSTRUCTION.md) and the
  Figure A1 description (README) aligned with the revised manuscript.

No coefficient, SE, p-value, or N changed. Validation: 136/136 pass.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/tables/table4_robustness_summary.xlsx
+++ b/results/tables/table4_robustness_summary.xlsx
@@ -22,43 +22,43 @@
     <t>key_finding</t>
   </si>
   <si>
-    <t>assessment</t>
+    <t>verdict</t>
   </si>
   <si>
     <t>Future-news placebo</t>
   </si>
   <si>
-    <t>NonDevRel placebo</t>
-  </si>
-  <si>
-    <t>Baseline alternative timing</t>
+    <t>Generic news placebo</t>
+  </si>
+  <si>
+    <t>Alternative timing_baseline</t>
+  </si>
+  <si>
+    <t>Alternative timing_crisis</t>
   </si>
   <si>
     <t>LOO sensitivity</t>
   </si>
   <si>
-    <t>Development vs. emergency alternative timing</t>
-  </si>
-  <si>
-    <t>Development vs. emergency crisis-type</t>
-  </si>
-  <si>
-    <t>Future media does not predict current ODA: gamma=0.048, p=0.144.</t>
-  </si>
-  <si>
-    <t>Development-related coverage predicts ODA (beta=0.084, p=0.035). Generic country coverage does not (beta=-0.019, p=0.556). 7 of 7 generic-coverage estimates are null.</t>
-  </si>
-  <si>
-    <t>The association remains positive for roughly three years, peaking contemporaneously before fading by year four (see alt_timing_baseline_results.csv).</t>
-  </si>
-  <si>
-    <t>No sign reversals in any analysis. Only the already-marginal 60-month rolling estimate (p=0.075 in the full sample) shows 6 significance flips (6/140).</t>
-  </si>
-  <si>
-    <t>See emergency_temporal_results.csv rows H4_within_emergency_contemporaneous / H4_within_emergency_forward for the contemporaneous-vs-forward-window comparison.</t>
-  </si>
-  <si>
-    <t>All 6 crisis types are individually positive and significant (p&lt;0.05); joint test: chi2(6)=28.06, p=9.168e-05.</t>
+    <t>Crisis-type heterogeneity</t>
+  </si>
+  <si>
+    <t>Future media does not predict current ODA: γ = 0.048, p = 0.144.</t>
+  </si>
+  <si>
+    <t>Generic country coverage does not predict ODA (β = -0.019, p = 0.556); same across all 7 temporal headlines.</t>
+  </si>
+  <si>
+    <t>The association remains positive for roughly three years, peaking contemporaneously before fading in year four.</t>
+  </si>
+  <si>
+    <t>Emergency ODA is associated with contemporaneous crisis coverage (β = 0.097, p = 0.009), but not previous news (p = 0.145).</t>
+  </si>
+  <si>
+    <t>No sign reversals in any analysis. Only the roll60 estimate shows six significance-status changes (6/140).</t>
+  </si>
+  <si>
+    <t>All 6 crisis types are individually positive and significant (p &lt; 0.05); joint test: χ²(6) = 28.06, p &lt; 0.001.</t>
   </si>
   <si>
     <t>Pass</t>

</xml_diff>

<commit_message>
Drop H4 top-1% trim from reported outputs; align Table 4/A4 with manuscript
- Table A4: H4 rows only (no trim row, no former-spec Panel B)
- Table 4: renamed timing rows, restored H4 estimator-sensitivity row,
  added H3 coverage-threshold row (data-driven from Table A6 results)
- Trim is still estimated in h4_common_exposure.py but no longer reported

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/tables/table4_robustness_summary.xlsx
+++ b/results/tables/table4_robustness_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>diagnostic</t>
   </si>
@@ -31,19 +31,22 @@
     <t>Generic news placebo</t>
   </si>
   <si>
-    <t>Alternative timing_baseline</t>
-  </si>
-  <si>
-    <t>Alternative timing_H4</t>
+    <t>Alternative timing (baseline)</t>
+  </si>
+  <si>
+    <t>Alternative timing (H4)</t>
   </si>
   <si>
     <t>LOO sensitivity</t>
   </si>
   <si>
-    <t>Influential observations_H4</t>
-  </si>
-  <si>
-    <t>Crisis-type heterogeneity (exploratory)</t>
+    <t>Coverage-threshold sensitivity (H3)</t>
+  </si>
+  <si>
+    <t>Estimator sensitivity (H4)</t>
+  </si>
+  <si>
+    <t>Crisis-type heterogeneity</t>
   </si>
   <si>
     <t>Future media does not predict current ODA: γ = 0.048, p = 0.144.</t>
@@ -61,7 +64,10 @@
     <t>No sign reversals in any analysis. Only the roll60 estimate shows six significance-status changes (6/140).</t>
   </si>
   <si>
-    <t>Top-1% trim of emergency commitments: β = 0.523, p = 0.007. A log(x+1) OLS counterpart does not reproduce the difference (β = 0.006, p = 0.864).</t>
+    <t>Streak estimates remain positive at every streak length for thresholds of 1–5 articles per month; at 10 articles the ≥ 60-month estimate is β = -0.032, p = 0.816.</t>
+  </si>
+  <si>
+    <t>A log(x+1) OLS counterpart of the stacked model does not reproduce the contemporaneous difference (β = 0.006, p = 0.864).</t>
   </si>
   <si>
     <t>All 6 crisis types are individually positive and significant (p &lt; 0.05); joint test: χ²(6) = 28.057, p &lt; 0.001.</t>
@@ -80,16 +86,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -105,7 +103,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -113,30 +111,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -431,17 +411,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -450,10 +430,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -461,10 +441,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -472,10 +452,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -483,10 +463,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -494,10 +474,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -505,10 +485,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -516,10 +496,21 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Non-development placebo: sports coverage replaces residual generic coverage
The generic placebo was built as (crisis-excluded country news) - DevRel,
clipped at 0, which removed DevRel x crisis-keyword articles twice. It is
replaced by a topically defined negative control: non-devrel sports
coverage of the same countries (BigKinds sports categories), counted from
the raw corpus with the devrel country detector
(topic_placebo_country_month.csv). Entertainment/celebrity counts are in
the file but not used (plausible affinity channel to aid).

All seven sports estimates are null (p = .18-.56); devrel estimates and
samples unchanged. Table A2, Table 4 and Figure 8 regenerated; validator
145/145.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/tables/table4_robustness_summary.xlsx
+++ b/results/tables/table4_robustness_summary.xlsx
@@ -28,7 +28,7 @@
     <t>Future-news placebo</t>
   </si>
   <si>
-    <t>Generic news placebo</t>
+    <t>Sports news placebo</t>
   </si>
   <si>
     <t>Alternative timing (baseline)</t>
@@ -52,7 +52,7 @@
     <t>Future media does not predict current ODA: γ = 0.048, p = 0.144.</t>
   </si>
   <si>
-    <t>Generic country coverage does not predict ODA (β = -0.019, p = 0.556); same across all 7 temporal headlines.</t>
+    <t>Sports coverage of the same countries does not predict ODA (β = 0.032, p = 0.183); same across all 7 temporal headlines.</t>
   </si>
   <si>
     <t>The association remains positive for roughly three years, peaking contemporaneously before fading in year four.</t>

</xml_diff>

<commit_message>
News-substance placebo: devrel vs. all country news vs. sports news
Each of the seven headline measures is now estimated with three media
series on one matched sample: development-relevant coverage, all news
mentioning the country (allnews_country_month.csv, any topic, devrel
included), and non-devrel sports coverage. DevRel is significant on 7/7,
all country news on 4/7 (smaller than DevRel on 6/7; larger only at
streak >= 60), sports on 0/7. Table A2, Table 4 and Figure 8 regenerated;
validator 147/147.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/tables/table4_robustness_summary.xlsx
+++ b/results/tables/table4_robustness_summary.xlsx
@@ -28,7 +28,7 @@
     <t>Future-news placebo</t>
   </si>
   <si>
-    <t>Sports news placebo</t>
+    <t>News-substance placebo</t>
   </si>
   <si>
     <t>Alternative timing (baseline)</t>
@@ -52,7 +52,7 @@
     <t>Future media does not predict current ODA: γ = 0.048, p = 0.144.</t>
   </si>
   <si>
-    <t>Sports coverage of the same countries does not predict ODA (β = 0.032, p = 0.183); same across all 7 temporal headlines.</t>
+    <t>DevRel coverage is significant (p &lt; 0.10) on 7/7 headline measures, all country news on 4/7, and sports news on 0/7; all news exceeds DevRel only at streak ≥ 60.</t>
   </si>
   <si>
     <t>The association remains positive for roughly three years, peaking contemporaneously before fading in year four.</t>

</xml_diff>

<commit_message>
Table 4: drop the Pass/Mixed verdict column; findings unchanged
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/tables/table4_robustness_summary.xlsx
+++ b/results/tables/table4_robustness_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>diagnostic</t>
   </si>
@@ -22,9 +22,6 @@
     <t>key_finding</t>
   </si>
   <si>
-    <t>verdict</t>
-  </si>
-  <si>
     <t>Future-news placebo</t>
   </si>
   <si>
@@ -71,15 +68,6 @@
   </si>
   <si>
     <t>All 6 crisis types are individually positive and significant (p &lt; 0.05); joint test: χ²(6) = 28.057, p &lt; 0.001.</t>
-  </si>
-  <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t>Mixed</t>
-  </si>
-  <si>
-    <t>—</t>
   </si>
 </sst>
 </file>
@@ -411,106 +399,79 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>15</v>
       </c>
-      <c r="C6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>16</v>
       </c>
-      <c r="C7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
         <v>9</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>17</v>
-      </c>
-      <c r="C8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>